<commit_message>
US03: refuse a past event date on submit; no mandatory fields
The customer never specified mandatory fields (Product Owner decision, 24 Oct 2026), so only a date that has already passed is refused. Removes TC-029 to TC-032 from the US03 test cases.
</commit_message>
<xml_diff>
--- a/docs/testing/US03_Create_Event_Request_Test_Cases.xlsx
+++ b/docs/testing/US03_Create_Event_Request_Test_Cases.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -703,17 +703,17 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>TC-029</t>
+          <t>TC-033</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Check missing mandatory event details are shown inline on step 1</t>
+          <t>Check an event date in the past cannot be entered</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Inline validation errors</t>
+          <t>No past event date</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -723,19 +723,19 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Picker greying verified through the min attribute rather than visually. Today's date accepted not separately checked.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>TC-030</t>
+          <t>TC-034</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Check missing venue and equipment details are shown inline on step 2</t>
+          <t>Check the registration closing date must be between today and the event date</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -750,24 +750,24 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Layout cannot be left blank in the UI: one option is always selected (Banquet by default). Run 08/10/2026 12:40-12:55 SGT.</t>
+          <t>Run 08/10/2026 12:40-12:55 SGT.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>TC-031</t>
+          <t>TC-035</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Check missing registration details are shown inline on step 3</t>
+          <t>Check a draft can be saved, reopened and saved again without creating a duplicate</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Inline validation errors</t>
+          <t>Event request saved</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -784,17 +784,17 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>TC-032</t>
+          <t>TC-036</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Check invalid values are rejected with inline errors</t>
+          <t>Check a submitted request is stored and still shown after a reload</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Inline validation errors</t>
+          <t>Event request saved</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -804,24 +804,24 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Run 08/10/2026 12:40-12:55 SGT.</t>
+          <t>Run 08/10/2026 12:40-12:55 SGT. Test data (events 1 and 2) was deleted from Supabase after the run.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>TC-033</t>
+          <t>TC-037</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Check an event date in the past cannot be entered</t>
+          <t>Check only Event Organisers can create event requests</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>No past event date</t>
+          <t>Organiser only</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -831,170 +831,62 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Picker greying verified through the min attribute rather than visually. Today's date accepted not separately checked.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>TC-034</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Check the registration closing date must be between today and the event date</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Inline validation errors</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
+          <t>Run 08/10/2026 12:40-12:55 SGT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Run 08/10/2026 12:40-12:55 SGT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>TC-035</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Check a draft can be saved, reopened and saved again without creating a duplicate</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Event request saved</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Run 08/10/2026 12:40-12:55 SGT.</t>
-        </is>
+      <c r="D15" s="8">
+        <f>COUNTIF($D$5:$D$13,"Pass")</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>TC-036</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Check a submitted request is stored and still shown after a reload</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Event request saved</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Run 08/10/2026 12:40-12:55 SGT. Test data (events 1 and 2) was deleted from Supabase after the run.</t>
-        </is>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D16" s="8">
+        <f>COUNTIF($D$5:$D$13,"Fail")</f>
+        <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>TC-037</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Check only Event Organisers can create event requests</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Organiser only</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Run 08/10/2026 12:40-12:55 SGT.</t>
-        </is>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="D17" s="8">
+        <f>COUNTIF($D$5:$D$13,"Not Executed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D18" s="8">
+        <f>COUNTIF($D$5:$D$13,"Blocked")</f>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="D19" s="8">
-        <f>COUNTIF($D$5:$D$17,"Pass")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="D20" s="8">
-        <f>COUNTIF($D$5:$D$17,"Fail")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="D21" s="8">
-        <f>COUNTIF($D$5:$D$17,"Not Executed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-      <c r="D22" s="8">
-        <f>COUNTIF($D$5:$D$17,"Blocked")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="C23" s="7" t="inlineStr">
-        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D23" s="7">
-        <f>SUM(D19:D22)</f>
+      <c r="D19" s="7">
+        <f>SUM(D15:D18)</f>
         <v/>
       </c>
     </row>
@@ -1013,7 +905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B222"/>
+  <dimension ref="A1:B154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1785,7 +1677,7 @@
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>TC-029</t>
+          <t>TC-033</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1689,7 @@
       </c>
       <c r="B74" s="13" t="inlineStr">
         <is>
-          <t>Check missing mandatory event details are shown inline on step 1</t>
+          <t>Check an event date in the past cannot be entered</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1705,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="28" customHeight="1">
+    <row r="76" ht="42" customHeight="1">
       <c r="A76" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1821,8 +1713,9 @@
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
-          <t>1. Leave every field on step 1 empty
-2. Click Continue</t>
+          <t>1. Open the Proposed date picker and try to choose yesterday
+2. Type yesterday's date into the field
+3. Complete the other steps and click Submit for review</t>
         </is>
       </c>
     </row>
@@ -1834,11 +1727,11 @@
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
-          <t>All step 1 fields empty</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="42" customHeight="1">
+          <t>Proposed date=yesterday's date</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="56" customHeight="1">
       <c r="A78" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1846,7 +1739,7 @@
       </c>
       <c r="B78" s="13" t="inlineStr">
         <is>
-          <t>Stays on step 1. Red messages appear under each field: 'Event name is required.', 'Event description is required.', 'Event type is required.', 'Preferred date is required.', 'Expected attendance must be a positive whole number.'</t>
+          <t>Step 1: dates before today are greyed out in the picker. Step 3: the request is not submitted and 'Preferred date cannot be in the past.' is shown. Today's date is accepted. (No other field is mandatory: Product Owner decision, 24 Oct 2026.)</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1787,7 @@
       </c>
       <c r="B82" s="16" t="inlineStr">
         <is>
-          <t>Continue on an empty Basics step showed an 'Outstanding mandatory fields' summary, red messages under name, description, type, preferred date and attendance, and the toast 'Complete the highlighted fields before continuing.'; the step did not advance.</t>
+          <t>The date input has min=2026-10-08 (today, local), so earlier dates cannot be picked. Typing 2026-01-15 and pressing Continue showed 'Preferred date cannot be in the past.' under the date and in the summary; the step did not advance.</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1803,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="15" customHeight="1">
+    <row r="84" ht="28" customHeight="1">
       <c r="A84" s="15" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -1918,7 +1811,7 @@
       </c>
       <c r="B84" s="16" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Picker greying verified through the min attribute rather than visually. Today's date accepted not separately checked.</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1859,7 @@
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
-          <t>TC-030</t>
+          <t>TC-034</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1871,7 @@
       </c>
       <c r="B91" s="13" t="inlineStr">
         <is>
-          <t>Check missing venue and equipment details are shown inline on step 2</t>
+          <t>Check the registration closing date must be between today and the event date</t>
         </is>
       </c>
     </row>
@@ -1990,744 +1883,17 @@
       </c>
       <c r="B92" s="13" t="inlineStr">
         <is>
-          <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Signed in as the Event Organiser. On New request, step 1 (Basics), with an empty form. Step 1 completed with valid details.</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="42" customHeight="1">
+          <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Signed in as the Event Organiser. On New request, step 1 (Basics), with an empty form. Steps 1-2 completed with the event 30 days from today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="56" customHeight="1">
       <c r="A93" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
       <c r="B93" s="13" t="inlineStr">
-        <is>
-          <t>1. On step 2 leave location and capacity empty
-2. Add 1 Projector but leave its technical requirements empty
-3. Click Continue</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="15" customHeight="1">
-      <c r="A94" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B94" s="13" t="inlineStr">
-        <is>
-          <t>Location=(empty); Capacity=(empty); Projector x1; Technical requirements=(empty)</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="28" customHeight="1">
-      <c r="A95" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B95" s="13" t="inlineStr">
-        <is>
-          <t>Stays on step 2. Inline errors: 'Venue location is required.', 'Venue capacity must be a positive whole number.', 'Equipment technical requirements are required.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="15" customHeight="1">
-      <c r="A96" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B96" s="13" t="inlineStr">
-        <is>
-          <t>Zhenhan</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="15" customHeight="1">
-      <c r="A97" s="12" t="inlineStr">
-        <is>
-          <t>Date of Creation</t>
-        </is>
-      </c>
-      <c r="B97" s="13" t="inlineStr">
-        <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="15" customHeight="1">
-      <c r="A98" s="14" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B98" s="14" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="56" customHeight="1">
-      <c r="A99" s="15" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B99" s="16" t="inlineStr">
-        <is>
-          <t>Blank venue location and blank capacity showed the 'Outstanding mandatory fields' summary plus 'Venue location is required.' and 'Venue capacity must be a positive whole number.' under each field; a Projector with blank technical requirements showed 'Equipment technical requirements are required.' under the projector row. The step did not advance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="15" customHeight="1">
-      <c r="A100" s="15" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B100" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="28" customHeight="1">
-      <c r="A101" s="15" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B101" s="16" t="inlineStr">
-        <is>
-          <t>Layout cannot be left blank in the UI: one option is always selected (Banquet by default). Run 08/10/2026 12:40-12:55 SGT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="15" customHeight="1">
-      <c r="A102" s="15" t="inlineStr">
-        <is>
-          <t>Executed By</t>
-        </is>
-      </c>
-      <c r="B102" s="16" t="inlineStr">
-        <is>
-          <t>Claude Code session spm-g5t8-d8 (for Zhenhan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="15" customHeight="1">
-      <c r="A103" s="15" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B103" s="16" t="inlineStr">
-        <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="15" customHeight="1">
-      <c r="A106" s="11" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B106" s="11" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="15" customHeight="1">
-      <c r="A107" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B107" s="13" t="inlineStr">
-        <is>
-          <t>TC-031</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="15" customHeight="1">
-      <c r="A108" s="12" t="inlineStr">
-        <is>
-          <t>Test Scenario</t>
-        </is>
-      </c>
-      <c r="B108" s="13" t="inlineStr">
-        <is>
-          <t>Check missing registration details are shown inline on step 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="42" customHeight="1">
-      <c r="A109" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B109" s="13" t="inlineStr">
-        <is>
-          <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Signed in as the Event Organiser. On New request, step 1 (Basics), with an empty form. Steps 1-2 completed with valid data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="42" customHeight="1">
-      <c r="A110" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B110" s="13" t="inlineStr">
-        <is>
-          <t>1. Tick Enable attendee registration
-2. Clear Registration cap and leave Registration closes empty
-3. Click Submit for review</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="15" customHeight="1">
-      <c r="A111" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B111" s="13" t="inlineStr">
-        <is>
-          <t>Registration cap=(empty); Registration closes=(empty)</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="28" customHeight="1">
-      <c r="A112" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B112" s="13" t="inlineStr">
-        <is>
-          <t>Request is not submitted. Inline errors: 'Registration capacity must be a positive whole number.', 'Registration closing date is required.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="15" customHeight="1">
-      <c r="A113" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B113" s="13" t="inlineStr">
-        <is>
-          <t>Zhenhan</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="15" customHeight="1">
-      <c r="A114" s="12" t="inlineStr">
-        <is>
-          <t>Date of Creation</t>
-        </is>
-      </c>
-      <c r="B114" s="13" t="inlineStr">
-        <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="15" customHeight="1">
-      <c r="A115" s="14" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B115" s="14" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="42" customHeight="1">
-      <c r="A116" s="15" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B116" s="16" t="inlineStr">
-        <is>
-          <t>Registration cap 0, and cap left blank, each showed 'Registration capacity must be a positive whole number.' under the cap field; a closing date after the event showed 'Registration must close on or before the event date.'. No API request was sent for any rejected submit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="15" customHeight="1">
-      <c r="A117" s="15" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B117" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="15" customHeight="1">
-      <c r="A118" s="15" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B118" s="16" t="inlineStr">
-        <is>
-          <t>Run 08/10/2026 12:40-12:55 SGT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="15" customHeight="1">
-      <c r="A119" s="15" t="inlineStr">
-        <is>
-          <t>Executed By</t>
-        </is>
-      </c>
-      <c r="B119" s="16" t="inlineStr">
-        <is>
-          <t>Claude Code session spm-g5t8-d8 (for Zhenhan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="15" customHeight="1">
-      <c r="A120" s="15" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B120" s="16" t="inlineStr">
-        <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="15" customHeight="1">
-      <c r="A123" s="11" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B123" s="11" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="15" customHeight="1">
-      <c r="A124" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B124" s="13" t="inlineStr">
-        <is>
-          <t>TC-032</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="15" customHeight="1">
-      <c r="A125" s="12" t="inlineStr">
-        <is>
-          <t>Test Scenario</t>
-        </is>
-      </c>
-      <c r="B125" s="13" t="inlineStr">
-        <is>
-          <t>Check invalid values are rejected with inline errors</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="28" customHeight="1">
-      <c r="A126" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B126" s="13" t="inlineStr">
-        <is>
-          <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Signed in as the Event Organiser. On New request, step 1 (Basics), with an empty form.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="28" customHeight="1">
-      <c r="A127" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B127" s="13" t="inlineStr">
-        <is>
-          <t>1. Enter valid details but Expected attendance=0 and End earlier than Start
-2. Click Continue</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" ht="28" customHeight="1">
-      <c r="A128" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B128" s="13" t="inlineStr">
-        <is>
-          <t>Name=Startup Pitch Night; Description=Eight student ventures pitch to investors; Type=Networking; Date=a date 30 days from today; Start=18:30; End=17:00; Expected attendance=0</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="28" customHeight="1">
-      <c r="A129" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B129" s="13" t="inlineStr">
-        <is>
-          <t>Stays on step 1. Inline errors: 'Expected attendance must be a positive whole number.', 'End time must be later than start time.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" ht="15" customHeight="1">
-      <c r="A130" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B130" s="13" t="inlineStr">
-        <is>
-          <t>Zhenhan</t>
-        </is>
-      </c>
-    </row>
-    <row r="131" ht="15" customHeight="1">
-      <c r="A131" s="12" t="inlineStr">
-        <is>
-          <t>Date of Creation</t>
-        </is>
-      </c>
-      <c r="B131" s="13" t="inlineStr">
-        <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" ht="15" customHeight="1">
-      <c r="A132" s="14" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B132" s="14" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="42" customHeight="1">
-      <c r="A133" s="15" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B133" s="16" t="inlineStr">
-        <is>
-          <t>Start 15:00 / end 14:00 and attendance 0 showed 'End time must be later than start time.' and 'Expected attendance must be a positive whole number.' under the fields and in the summary; the step did not advance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" ht="15" customHeight="1">
-      <c r="A134" s="15" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B134" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="15" customHeight="1">
-      <c r="A135" s="15" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B135" s="16" t="inlineStr">
-        <is>
-          <t>Run 08/10/2026 12:40-12:55 SGT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="136" ht="15" customHeight="1">
-      <c r="A136" s="15" t="inlineStr">
-        <is>
-          <t>Executed By</t>
-        </is>
-      </c>
-      <c r="B136" s="16" t="inlineStr">
-        <is>
-          <t>Claude Code session spm-g5t8-d8 (for Zhenhan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="137" ht="15" customHeight="1">
-      <c r="A137" s="15" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B137" s="16" t="inlineStr">
-        <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="15" customHeight="1">
-      <c r="A140" s="11" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B140" s="11" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="15" customHeight="1">
-      <c r="A141" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B141" s="13" t="inlineStr">
-        <is>
-          <t>TC-033</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="15" customHeight="1">
-      <c r="A142" s="12" t="inlineStr">
-        <is>
-          <t>Test Scenario</t>
-        </is>
-      </c>
-      <c r="B142" s="13" t="inlineStr">
-        <is>
-          <t>Check an event date in the past cannot be entered</t>
-        </is>
-      </c>
-    </row>
-    <row r="143" ht="28" customHeight="1">
-      <c r="A143" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B143" s="13" t="inlineStr">
-        <is>
-          <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Signed in as the Event Organiser. On New request, step 1 (Basics), with an empty form.</t>
-        </is>
-      </c>
-    </row>
-    <row r="144" ht="42" customHeight="1">
-      <c r="A144" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B144" s="13" t="inlineStr">
-        <is>
-          <t>1. Open the Proposed date picker and try to choose yesterday
-2. Type yesterday's date into the field
-3. Complete the other step 1 fields and click Continue</t>
-        </is>
-      </c>
-    </row>
-    <row r="145" ht="15" customHeight="1">
-      <c r="A145" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B145" s="13" t="inlineStr">
-        <is>
-          <t>Proposed date=yesterday's date</t>
-        </is>
-      </c>
-    </row>
-    <row r="146" ht="28" customHeight="1">
-      <c r="A146" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B146" s="13" t="inlineStr">
-        <is>
-          <t>Step 1: dates before today are greyed out in the picker. Step 3: stays on step 1 with inline error 'Preferred date cannot be in the past.' Today's date is accepted</t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="15" customHeight="1">
-      <c r="A147" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B147" s="13" t="inlineStr">
-        <is>
-          <t>Zhenhan</t>
-        </is>
-      </c>
-    </row>
-    <row r="148" ht="15" customHeight="1">
-      <c r="A148" s="12" t="inlineStr">
-        <is>
-          <t>Date of Creation</t>
-        </is>
-      </c>
-      <c r="B148" s="13" t="inlineStr">
-        <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="15" customHeight="1">
-      <c r="A149" s="14" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B149" s="14" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="150" ht="42" customHeight="1">
-      <c r="A150" s="15" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B150" s="16" t="inlineStr">
-        <is>
-          <t>The date input has min=2026-10-08 (today, local), so earlier dates cannot be picked. Typing 2026-01-15 and pressing Continue showed 'Preferred date cannot be in the past.' under the date and in the summary; the step did not advance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="15" customHeight="1">
-      <c r="A151" s="15" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B151" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="28" customHeight="1">
-      <c r="A152" s="15" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B152" s="16" t="inlineStr">
-        <is>
-          <t>Picker greying verified through the min attribute rather than visually. Today's date accepted not separately checked.</t>
-        </is>
-      </c>
-    </row>
-    <row r="153" ht="15" customHeight="1">
-      <c r="A153" s="15" t="inlineStr">
-        <is>
-          <t>Executed By</t>
-        </is>
-      </c>
-      <c r="B153" s="16" t="inlineStr">
-        <is>
-          <t>Claude Code session spm-g5t8-d8 (for Zhenhan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="154" ht="15" customHeight="1">
-      <c r="A154" s="15" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B154" s="16" t="inlineStr">
-        <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="157" ht="15" customHeight="1">
-      <c r="A157" s="11" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B157" s="11" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="158" ht="15" customHeight="1">
-      <c r="A158" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B158" s="13" t="inlineStr">
-        <is>
-          <t>TC-034</t>
-        </is>
-      </c>
-    </row>
-    <row r="159" ht="15" customHeight="1">
-      <c r="A159" s="12" t="inlineStr">
-        <is>
-          <t>Test Scenario</t>
-        </is>
-      </c>
-      <c r="B159" s="13" t="inlineStr">
-        <is>
-          <t>Check the registration closing date must be between today and the event date</t>
-        </is>
-      </c>
-    </row>
-    <row r="160" ht="42" customHeight="1">
-      <c r="A160" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B160" s="13" t="inlineStr">
-        <is>
-          <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Signed in as the Event Organiser. On New request, step 1 (Basics), with an empty form. Steps 1-2 completed with the event 30 days from today.</t>
-        </is>
-      </c>
-    </row>
-    <row r="161" ht="56" customHeight="1">
-      <c r="A161" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B161" s="13" t="inlineStr">
         <is>
           <t>1. Tick Enable attendee registration, cap 120
 2. Set Registration closes to yesterday, click Submit for review
@@ -2736,181 +1902,181 @@
         </is>
       </c>
     </row>
-    <row r="162" ht="15" customHeight="1">
-      <c r="A162" s="12" t="inlineStr">
+    <row r="94" ht="15" customHeight="1">
+      <c r="A94" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B162" s="13" t="inlineStr">
+      <c r="B94" s="13" t="inlineStr">
         <is>
           <t>Registration closes=yesterday / event date + 1 day / event date</t>
         </is>
       </c>
     </row>
-    <row r="163" ht="42" customHeight="1">
-      <c r="A163" s="12" t="inlineStr">
+    <row r="95" ht="42" customHeight="1">
+      <c r="A95" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B163" s="13" t="inlineStr">
+      <c r="B95" s="13" t="inlineStr">
         <is>
           <t>Step 2: 'Registration closing date cannot be in the past.' Step 3: 'Registration must close on or before the event date.' Step 4: request is submitted (closing on the event day is allowed). The date picker only offers today to the event date</t>
         </is>
       </c>
     </row>
-    <row r="164" ht="15" customHeight="1">
-      <c r="A164" s="12" t="inlineStr">
+    <row r="96" ht="15" customHeight="1">
+      <c r="A96" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B164" s="13" t="inlineStr">
+      <c r="B96" s="13" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
-    <row r="165" ht="15" customHeight="1">
-      <c r="A165" s="12" t="inlineStr">
+    <row r="97" ht="15" customHeight="1">
+      <c r="A97" s="12" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B165" s="13" t="inlineStr">
+      <c r="B97" s="13" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
-    <row r="166" ht="15" customHeight="1">
-      <c r="A166" s="14" t="inlineStr">
+    <row r="98" ht="15" customHeight="1">
+      <c r="A98" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B166" s="14" t="inlineStr">
+      <c r="B98" s="14" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
-    <row r="167" ht="56" customHeight="1">
-      <c r="A167" s="15" t="inlineStr">
+    <row r="99" ht="56" customHeight="1">
+      <c r="A99" s="15" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B167" s="16" t="inlineStr">
+      <c r="B99" s="16" t="inlineStr">
         <is>
           <t>Past closing date (2026-10-01) showed 'Registration closing date cannot be in the past.'; a closing date after the event was rejected with 'Registration must close on or before the event date.'; a closing date on the event day (2026-12-01 for a 2026-12-01 event) was accepted and the request submitted (PUT /api/events/2 200). The picker offers only today to the event date.</t>
         </is>
       </c>
     </row>
-    <row r="168" ht="15" customHeight="1">
-      <c r="A168" s="15" t="inlineStr">
+    <row r="100" ht="15" customHeight="1">
+      <c r="A100" s="15" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B168" s="5" t="inlineStr">
+      <c r="B100" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
     </row>
-    <row r="169" ht="15" customHeight="1">
-      <c r="A169" s="15" t="inlineStr">
+    <row r="101" ht="15" customHeight="1">
+      <c r="A101" s="15" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B169" s="16" t="inlineStr">
+      <c r="B101" s="16" t="inlineStr">
         <is>
           <t>Run 08/10/2026 12:40-12:55 SGT.</t>
         </is>
       </c>
     </row>
-    <row r="170" ht="15" customHeight="1">
-      <c r="A170" s="15" t="inlineStr">
+    <row r="102" ht="15" customHeight="1">
+      <c r="A102" s="15" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
       </c>
-      <c r="B170" s="16" t="inlineStr">
+      <c r="B102" s="16" t="inlineStr">
         <is>
           <t>Claude Code session spm-g5t8-d8 (for Zhenhan)</t>
         </is>
       </c>
     </row>
-    <row r="171" ht="15" customHeight="1">
-      <c r="A171" s="15" t="inlineStr">
+    <row r="103" ht="15" customHeight="1">
+      <c r="A103" s="15" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B171" s="16" t="inlineStr">
+      <c r="B103" s="16" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
     </row>
-    <row r="174" ht="15" customHeight="1">
-      <c r="A174" s="11" t="inlineStr">
+    <row r="106" ht="15" customHeight="1">
+      <c r="A106" s="11" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B174" s="11" t="inlineStr">
+      <c r="B106" s="11" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
-    <row r="175" ht="15" customHeight="1">
-      <c r="A175" s="12" t="inlineStr">
+    <row r="107" ht="15" customHeight="1">
+      <c r="A107" s="12" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B175" s="13" t="inlineStr">
+      <c r="B107" s="13" t="inlineStr">
         <is>
           <t>TC-035</t>
         </is>
       </c>
     </row>
-    <row r="176" ht="15" customHeight="1">
-      <c r="A176" s="12" t="inlineStr">
+    <row r="108" ht="15" customHeight="1">
+      <c r="A108" s="12" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B176" s="13" t="inlineStr">
+      <c r="B108" s="13" t="inlineStr">
         <is>
           <t>Check a draft can be saved, reopened and saved again without creating a duplicate</t>
         </is>
       </c>
     </row>
-    <row r="177" ht="28" customHeight="1">
-      <c r="A177" s="12" t="inlineStr">
+    <row r="109" ht="28" customHeight="1">
+      <c r="A109" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B177" s="13" t="inlineStr">
+      <c r="B109" s="13" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Signed in as the Event Organiser. On New request, step 1 (Basics), with an empty form.</t>
         </is>
       </c>
     </row>
-    <row r="178" ht="56" customHeight="1">
-      <c r="A178" s="12" t="inlineStr">
+    <row r="110" ht="56" customHeight="1">
+      <c r="A110" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B178" s="13" t="inlineStr">
+      <c r="B110" s="13" t="inlineStr">
         <is>
           <t>1. Enter only Event name and click Save as draft
 2. On My events note the draft count, open the draft
@@ -2919,181 +2085,181 @@
         </is>
       </c>
     </row>
-    <row r="179" ht="15" customHeight="1">
-      <c r="A179" s="12" t="inlineStr">
+    <row r="111" ht="15" customHeight="1">
+      <c r="A111" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B179" s="13" t="inlineStr">
+      <c r="B111" s="13" t="inlineStr">
         <is>
           <t>Event name=Postgrad Welcome Drinks; Description=added in step 3</t>
         </is>
       </c>
     </row>
-    <row r="180" ht="42" customHeight="1">
-      <c r="A180" s="12" t="inlineStr">
+    <row r="112" ht="42" customHeight="1">
+      <c r="A112" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B180" s="13" t="inlineStr">
+      <c r="B112" s="13" t="inlineStr">
         <is>
           <t>Draft appears on My events with its name; reopening shows the saved values. After step 3 there is still ONE draft with the new description (no duplicate). After refresh the draft is still listed</t>
         </is>
       </c>
     </row>
-    <row r="181" ht="15" customHeight="1">
-      <c r="A181" s="12" t="inlineStr">
+    <row r="113" ht="15" customHeight="1">
+      <c r="A113" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B181" s="13" t="inlineStr">
+      <c r="B113" s="13" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
-    <row r="182" ht="15" customHeight="1">
-      <c r="A182" s="12" t="inlineStr">
+    <row r="114" ht="15" customHeight="1">
+      <c r="A114" s="12" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B182" s="13" t="inlineStr">
+      <c r="B114" s="13" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
-    <row r="183" ht="15" customHeight="1">
-      <c r="A183" s="14" t="inlineStr">
+    <row r="115" ht="15" customHeight="1">
+      <c r="A115" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B183" s="14" t="inlineStr">
+      <c r="B115" s="14" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
-    <row r="184" ht="42" customHeight="1">
-      <c r="A184" s="15" t="inlineStr">
+    <row r="116" ht="42" customHeight="1">
+      <c r="A116" s="15" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B184" s="16" t="inlineStr">
+      <c r="B116" s="16" t="inlineStr">
         <is>
           <t>New draft saved (POST 201, EVT-2) and listed on My events; reopened with all values restored on all 3 steps; renamed and saved as draft again -&gt; PUT /api/events/2 200 (no new POST). After a refresh My events showed EVT-2 with the new name and no EVT-3; Supabase had exactly 2 rows.</t>
         </is>
       </c>
     </row>
-    <row r="185" ht="15" customHeight="1">
-      <c r="A185" s="15" t="inlineStr">
+    <row r="117" ht="15" customHeight="1">
+      <c r="A117" s="15" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B185" s="5" t="inlineStr">
+      <c r="B117" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
     </row>
-    <row r="186" ht="15" customHeight="1">
-      <c r="A186" s="15" t="inlineStr">
+    <row r="118" ht="15" customHeight="1">
+      <c r="A118" s="15" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B186" s="16" t="inlineStr">
+      <c r="B118" s="16" t="inlineStr">
         <is>
           <t>Run 08/10/2026 12:40-12:55 SGT.</t>
         </is>
       </c>
     </row>
-    <row r="187" ht="15" customHeight="1">
-      <c r="A187" s="15" t="inlineStr">
+    <row r="119" ht="15" customHeight="1">
+      <c r="A119" s="15" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
       </c>
-      <c r="B187" s="16" t="inlineStr">
+      <c r="B119" s="16" t="inlineStr">
         <is>
           <t>Claude Code session spm-g5t8-d8 (for Zhenhan)</t>
         </is>
       </c>
     </row>
-    <row r="188" ht="15" customHeight="1">
-      <c r="A188" s="15" t="inlineStr">
+    <row r="120" ht="15" customHeight="1">
+      <c r="A120" s="15" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B188" s="16" t="inlineStr">
+      <c r="B120" s="16" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
     </row>
-    <row r="191" ht="15" customHeight="1">
-      <c r="A191" s="11" t="inlineStr">
+    <row r="123" ht="15" customHeight="1">
+      <c r="A123" s="11" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B191" s="11" t="inlineStr">
+      <c r="B123" s="11" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
-    <row r="192" ht="15" customHeight="1">
-      <c r="A192" s="12" t="inlineStr">
+    <row r="124" ht="15" customHeight="1">
+      <c r="A124" s="12" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B192" s="13" t="inlineStr">
+      <c r="B124" s="13" t="inlineStr">
         <is>
           <t>TC-036</t>
         </is>
       </c>
     </row>
-    <row r="193" ht="15" customHeight="1">
-      <c r="A193" s="12" t="inlineStr">
+    <row r="125" ht="15" customHeight="1">
+      <c r="A125" s="12" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B193" s="13" t="inlineStr">
+      <c r="B125" s="13" t="inlineStr">
         <is>
           <t>Check a submitted request is stored and still shown after a reload</t>
         </is>
       </c>
     </row>
-    <row r="194" ht="28" customHeight="1">
-      <c r="A194" s="12" t="inlineStr">
+    <row r="126" ht="28" customHeight="1">
+      <c r="A126" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B194" s="13" t="inlineStr">
+      <c r="B126" s="13" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Signed in as the Event Organiser. On New request, step 1 (Basics), with an empty form.</t>
         </is>
       </c>
     </row>
-    <row r="195" ht="42" customHeight="1">
-      <c r="A195" s="12" t="inlineStr">
+    <row r="127" ht="42" customHeight="1">
+      <c r="A127" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B195" s="13" t="inlineStr">
+      <c r="B127" s="13" t="inlineStr">
         <is>
           <t>1. Complete steps 1-3 with valid data (TC-025 to TC-028)
 2. Click Submit for review
@@ -3101,302 +2267,302 @@
         </is>
       </c>
     </row>
-    <row r="196" ht="42" customHeight="1">
-      <c r="A196" s="12" t="inlineStr">
+    <row r="128" ht="42" customHeight="1">
+      <c r="A128" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B196" s="13" t="inlineStr">
+      <c r="B128" s="13" t="inlineStr">
         <is>
           <t>Name=Startup Pitch Night; Description=Eight student ventures pitch to investors; Type=Networking; Date=a date 30 days from today; Start=18:30; End=21:00; Expected attendance=95; venue/equipment/registration as TC-026 to TC-028</t>
         </is>
       </c>
     </row>
-    <row r="197" ht="28" customHeight="1">
-      <c r="A197" s="12" t="inlineStr">
+    <row r="129" ht="28" customHeight="1">
+      <c r="A129" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B197" s="13" t="inlineStr">
+      <c r="B129" s="13" t="inlineStr">
         <is>
           <t>Confirmation 'Startup Pitch Night submitted for review.'; My events lists it as Submitted; it is still listed after refresh</t>
         </is>
       </c>
     </row>
-    <row r="198" ht="15" customHeight="1">
-      <c r="A198" s="12" t="inlineStr">
+    <row r="130" ht="15" customHeight="1">
+      <c r="A130" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B198" s="13" t="inlineStr">
+      <c r="B130" s="13" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
-    <row r="199" ht="15" customHeight="1">
-      <c r="A199" s="12" t="inlineStr">
+    <row r="131" ht="15" customHeight="1">
+      <c r="A131" s="12" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B199" s="13" t="inlineStr">
+      <c r="B131" s="13" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
-    <row r="200" ht="15" customHeight="1">
-      <c r="A200" s="14" t="inlineStr">
+    <row r="132" ht="15" customHeight="1">
+      <c r="A132" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B200" s="14" t="inlineStr">
+      <c r="B132" s="14" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
-    <row r="201" ht="42" customHeight="1">
-      <c r="A201" s="15" t="inlineStr">
+    <row r="133" ht="42" customHeight="1">
+      <c r="A133" s="15" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B201" s="16" t="inlineStr">
+      <c r="B133" s="16" t="inlineStr">
         <is>
           <t>EVT-2 submitted for review -&gt; PUT /api/events/2 200, toast '... submitted for review.', listed as Submitted on My events and still listed as Submitted after a page refresh. Supabase row: status submitted, submitted_at set.</t>
         </is>
       </c>
     </row>
-    <row r="202" ht="15" customHeight="1">
-      <c r="A202" s="15" t="inlineStr">
+    <row r="134" ht="15" customHeight="1">
+      <c r="A134" s="15" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B202" s="5" t="inlineStr">
+      <c r="B134" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
     </row>
-    <row r="203" ht="28" customHeight="1">
-      <c r="A203" s="15" t="inlineStr">
+    <row r="135" ht="28" customHeight="1">
+      <c r="A135" s="15" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B203" s="16" t="inlineStr">
+      <c r="B135" s="16" t="inlineStr">
         <is>
           <t>Run 08/10/2026 12:40-12:55 SGT. Test data (events 1 and 2) was deleted from Supabase after the run.</t>
         </is>
       </c>
     </row>
-    <row r="204" ht="15" customHeight="1">
-      <c r="A204" s="15" t="inlineStr">
+    <row r="136" ht="15" customHeight="1">
+      <c r="A136" s="15" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
       </c>
-      <c r="B204" s="16" t="inlineStr">
+      <c r="B136" s="16" t="inlineStr">
         <is>
           <t>Claude Code session spm-g5t8-d8 (for Zhenhan)</t>
         </is>
       </c>
     </row>
-    <row r="205" ht="15" customHeight="1">
-      <c r="A205" s="15" t="inlineStr">
+    <row r="137" ht="15" customHeight="1">
+      <c r="A137" s="15" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B205" s="16" t="inlineStr">
+      <c r="B137" s="16" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
     </row>
-    <row r="208" ht="15" customHeight="1">
-      <c r="A208" s="11" t="inlineStr">
+    <row r="140" ht="15" customHeight="1">
+      <c r="A140" s="11" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B208" s="11" t="inlineStr">
+      <c r="B140" s="11" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
-    <row r="209" ht="15" customHeight="1">
-      <c r="A209" s="12" t="inlineStr">
+    <row r="141" ht="15" customHeight="1">
+      <c r="A141" s="12" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B209" s="13" t="inlineStr">
+      <c r="B141" s="13" t="inlineStr">
         <is>
           <t>TC-037</t>
         </is>
       </c>
     </row>
-    <row r="210" ht="15" customHeight="1">
-      <c r="A210" s="12" t="inlineStr">
+    <row r="142" ht="15" customHeight="1">
+      <c r="A142" s="12" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B210" s="13" t="inlineStr">
+      <c r="B142" s="13" t="inlineStr">
         <is>
           <t>Check only Event Organisers can create event requests</t>
         </is>
       </c>
     </row>
-    <row r="211" ht="15" customHeight="1">
-      <c r="A211" s="12" t="inlineStr">
+    <row r="143" ht="15" customHeight="1">
+      <c r="A143" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B211" s="13" t="inlineStr">
+      <c r="B143" s="13" t="inlineStr">
         <is>
           <t>App running. Signed in as the Attendee.</t>
         </is>
       </c>
     </row>
-    <row r="212" ht="42" customHeight="1">
-      <c r="A212" s="12" t="inlineStr">
+    <row r="144" ht="42" customHeight="1">
+      <c r="A144" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B212" s="13" t="inlineStr">
+      <c r="B144" s="13" t="inlineStr">
         <is>
           <t>1. Type http://localhost:3000/new-request in the address bar
 2. DevTools &gt; Console: fetch('/api/events',{method:'POST',headers:{'Content-Type':'application/json'},body:'{"name":"x"}'}).then(r=&gt;r.status)</t>
         </is>
       </c>
     </row>
-    <row r="213" ht="15" customHeight="1">
-      <c r="A213" s="12" t="inlineStr">
+    <row r="145" ht="15" customHeight="1">
+      <c r="A145" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B213" s="13" t="inlineStr">
+      <c r="B145" s="13" t="inlineStr">
         <is>
           <t>Email=sam.adeyemi@student.connectsphere.edu; Password=&lt;team password&gt;</t>
         </is>
       </c>
     </row>
-    <row r="214" ht="28" customHeight="1">
-      <c r="A214" s="12" t="inlineStr">
+    <row r="146" ht="28" customHeight="1">
+      <c r="A146" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B214" s="13" t="inlineStr">
+      <c r="B146" s="13" t="inlineStr">
         <is>
           <t>Step 1: redirected to Browse events with 'You don't have permission to view that page.' Step 2: returns 403; nothing is created</t>
         </is>
       </c>
     </row>
-    <row r="215" ht="15" customHeight="1">
-      <c r="A215" s="12" t="inlineStr">
+    <row r="147" ht="15" customHeight="1">
+      <c r="A147" s="12" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B215" s="13" t="inlineStr">
+      <c r="B147" s="13" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
-    <row r="216" ht="15" customHeight="1">
-      <c r="A216" s="12" t="inlineStr">
+    <row r="148" ht="15" customHeight="1">
+      <c r="A148" s="12" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B216" s="13" t="inlineStr">
+      <c r="B148" s="13" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
-    <row r="217" ht="15" customHeight="1">
-      <c r="A217" s="14" t="inlineStr">
+    <row r="149" ht="15" customHeight="1">
+      <c r="A149" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B217" s="14" t="inlineStr">
+      <c r="B149" s="14" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
-    <row r="218" ht="56" customHeight="1">
-      <c r="A218" s="15" t="inlineStr">
+    <row r="150" ht="56" customHeight="1">
+      <c r="A150" s="15" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B218" s="16" t="inlineStr">
+      <c r="B150" s="16" t="inlineStr">
         <is>
           <t>Signed in as Sam Adeyemi (attendee): sidebar shows only Browse events; opening /new-request redirected to /browse with 'You don't have permission to view that page.'; POST /api/events from the attendee session returned 403 'You don't have permission to do that' and no row was created. The submitted test events were not shown on Browse (not published).</t>
         </is>
       </c>
     </row>
-    <row r="219" ht="15" customHeight="1">
-      <c r="A219" s="15" t="inlineStr">
+    <row r="151" ht="15" customHeight="1">
+      <c r="A151" s="15" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B219" s="5" t="inlineStr">
+      <c r="B151" s="5" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
     </row>
-    <row r="220" ht="15" customHeight="1">
-      <c r="A220" s="15" t="inlineStr">
+    <row r="152" ht="15" customHeight="1">
+      <c r="A152" s="15" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B220" s="16" t="inlineStr">
+      <c r="B152" s="16" t="inlineStr">
         <is>
           <t>Run 08/10/2026 12:40-12:55 SGT.</t>
         </is>
       </c>
     </row>
-    <row r="221" ht="15" customHeight="1">
-      <c r="A221" s="15" t="inlineStr">
+    <row r="153" ht="15" customHeight="1">
+      <c r="A153" s="15" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
       </c>
-      <c r="B221" s="16" t="inlineStr">
+      <c r="B153" s="16" t="inlineStr">
         <is>
           <t>Claude Code session spm-g5t8-d8 (for Zhenhan)</t>
         </is>
       </c>
     </row>
-    <row r="222" ht="15" customHeight="1">
-      <c r="A222" s="15" t="inlineStr">
+    <row r="154" ht="15" customHeight="1">
+      <c r="A154" s="15" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B222" s="16" t="inlineStr">
+      <c r="B154" s="16" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>

</xml_diff>